<commit_message>
stop camera, logo, label,
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +461,58 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>total_time_present</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2023130344</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>kent</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>45841.9600859838</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>45841.97639271991</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>LATE</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0 days 00:23:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>kent</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>45841.97702189815</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>45841.97736334491</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>LATE</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0 days 00:00:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
12 hour format, register, change password, move reset button, admin settings layout
</commit_message>
<xml_diff>
--- a/attendance.xlsx
+++ b/attendance.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,7 +466,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2023130344</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -474,45 +474,19 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>45841.9600859838</v>
+        <v>45842.03369025463</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>45841.97639271991</v>
+        <v>45842.03392194444</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>LATE</t>
+          <t>PRESENT</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0 days 00:23:28</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>kent</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>45841.97702189815</v>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>45841.97736334491</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>LATE</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>0 days 00:00:29</t>
+          <t>0 days 00:00:20</t>
         </is>
       </c>
     </row>

</xml_diff>